<commit_message>
Remove emissions per capita and add emissions change. Update dataset and all supplementary tables and figures.
</commit_message>
<xml_diff>
--- a/Output data/Latest data point per country-indicator.xlsx
+++ b/Output data/Latest data point per country-indicator.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Food system emissions per capita</t>
+          <t>Food system emissions change</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -1522,6 +1522,11 @@
           <t>2022</t>
         </is>
       </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="AC5" t="inlineStr">
         <is>
           <t>2022</t>
@@ -1664,7 +1669,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1890,7 +1895,7 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -2083,7 +2088,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -2361,7 +2366,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -2610,7 +2615,7 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -2830,7 +2835,7 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
@@ -3098,7 +3103,7 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
@@ -3317,7 +3322,7 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
@@ -3485,7 +3490,7 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -3720,7 +3725,7 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -3954,7 +3959,7 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -4162,7 +4167,7 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -4390,7 +4395,7 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -4623,7 +4628,7 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -4886,7 +4891,7 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -5138,7 +5143,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -5393,7 +5398,7 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -5670,7 +5675,7 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -5934,7 +5939,7 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -6218,7 +6223,7 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -6442,7 +6447,7 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -6630,7 +6635,7 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -6913,7 +6918,7 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
@@ -7175,7 +7180,7 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
@@ -7403,7 +7408,7 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
@@ -7669,7 +7674,7 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
@@ -7956,7 +7961,7 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
@@ -8198,7 +8203,7 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
@@ -8436,7 +8441,7 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
@@ -8684,7 +8689,7 @@
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
@@ -8951,7 +8956,7 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
@@ -9240,7 +9245,7 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
@@ -9514,7 +9519,7 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
@@ -9801,7 +9806,7 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
@@ -10100,7 +10105,7 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
@@ -10377,7 +10382,7 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
@@ -10671,7 +10676,7 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
@@ -10923,7 +10928,7 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
@@ -11151,7 +11156,7 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
@@ -11361,7 +11366,7 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
@@ -11579,7 +11584,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
@@ -11802,7 +11807,7 @@
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
@@ -12027,7 +12032,7 @@
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X48" t="inlineStr">
@@ -12274,7 +12279,7 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
@@ -12497,7 +12502,7 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
@@ -12713,7 +12718,7 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X51" t="inlineStr">
@@ -12951,7 +12956,7 @@
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
@@ -13243,7 +13248,7 @@
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
@@ -13540,7 +13545,7 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
@@ -13789,7 +13794,7 @@
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
@@ -14000,7 +14005,7 @@
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
@@ -14150,7 +14155,7 @@
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
@@ -14347,7 +14352,7 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
@@ -14580,7 +14585,7 @@
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
@@ -14876,7 +14881,7 @@
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
@@ -15138,7 +15143,7 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
@@ -15361,7 +15366,7 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
@@ -15579,7 +15584,7 @@
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X63" t="inlineStr">
@@ -15780,6 +15785,11 @@
           <t>2022</t>
         </is>
       </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="X64" t="inlineStr">
         <is>
           <t>2006</t>
@@ -15937,7 +15947,7 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X65" t="inlineStr">
@@ -16176,7 +16186,7 @@
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X66" t="inlineStr">
@@ -16447,7 +16457,7 @@
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X67" t="inlineStr">
@@ -16701,7 +16711,7 @@
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X68" t="inlineStr">
@@ -16979,7 +16989,7 @@
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X69" t="inlineStr">
@@ -17268,7 +17278,7 @@
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X70" t="inlineStr">
@@ -17497,7 +17507,7 @@
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X71" t="inlineStr">
@@ -17725,7 +17735,7 @@
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X72" t="inlineStr">
@@ -18007,7 +18017,7 @@
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X73" t="inlineStr">
@@ -18264,7 +18274,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X74" t="inlineStr">
@@ -18510,7 +18520,7 @@
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X75" t="inlineStr">
@@ -18735,7 +18745,7 @@
       </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X76" t="inlineStr">
@@ -19011,7 +19021,7 @@
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X77" t="inlineStr">
@@ -19268,7 +19278,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X78" t="inlineStr">
@@ -19501,7 +19511,7 @@
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X79" t="inlineStr">
@@ -19749,7 +19759,7 @@
       </c>
       <c r="W80" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr">
@@ -20033,7 +20043,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X81" t="inlineStr">
@@ -20327,7 +20337,7 @@
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X82" t="inlineStr">
@@ -20591,7 +20601,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X83" t="inlineStr">
@@ -20828,7 +20838,7 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X84" t="inlineStr">
@@ -21081,7 +21091,7 @@
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X85" t="inlineStr">
@@ -21300,7 +21310,7 @@
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X86" t="inlineStr">
@@ -21533,7 +21543,7 @@
       </c>
       <c r="W87" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X87" t="inlineStr">
@@ -21766,7 +21776,7 @@
       </c>
       <c r="W88" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X88" t="inlineStr">
@@ -22024,7 +22034,7 @@
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X89" t="inlineStr">
@@ -22316,7 +22326,7 @@
       </c>
       <c r="W90" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X90" t="inlineStr">
@@ -22580,7 +22590,7 @@
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X91" t="inlineStr">
@@ -22822,7 +22832,7 @@
       </c>
       <c r="W92" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="Z92" t="inlineStr">
@@ -23000,7 +23010,7 @@
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X93" t="inlineStr">
@@ -23238,7 +23248,7 @@
       </c>
       <c r="W94" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X94" t="inlineStr">
@@ -23522,7 +23532,7 @@
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X95" t="inlineStr">
@@ -23759,7 +23769,7 @@
       </c>
       <c r="W96" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X96" t="inlineStr">
@@ -24027,7 +24037,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X97" t="inlineStr">
@@ -24269,7 +24279,7 @@
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X98" t="inlineStr">
@@ -24545,7 +24555,7 @@
       </c>
       <c r="W99" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X99" t="inlineStr">
@@ -24799,7 +24809,7 @@
       </c>
       <c r="W100" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X100" t="inlineStr">
@@ -24974,6 +24984,11 @@
           <t>2022</t>
         </is>
       </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="AC101" t="inlineStr">
         <is>
           <t>2022</t>
@@ -25098,7 +25113,7 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X102" t="inlineStr">
@@ -25331,7 +25346,7 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X103" t="inlineStr">
@@ -25594,7 +25609,7 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X104" t="inlineStr">
@@ -25896,7 +25911,7 @@
       </c>
       <c r="W105" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X105" t="inlineStr">
@@ -26183,7 +26198,7 @@
       </c>
       <c r="W106" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X106" t="inlineStr">
@@ -26417,7 +26432,7 @@
       </c>
       <c r="W107" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="Y107" t="inlineStr">
@@ -26655,7 +26670,7 @@
       </c>
       <c r="W108" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X108" t="inlineStr">
@@ -26902,7 +26917,7 @@
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X109" t="inlineStr">
@@ -27085,7 +27100,7 @@
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="AC110" t="inlineStr">
@@ -27277,7 +27292,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X111" t="inlineStr">
@@ -27529,7 +27544,7 @@
       </c>
       <c r="W112" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X112" t="inlineStr">
@@ -27787,7 +27802,7 @@
       </c>
       <c r="W113" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X113" t="inlineStr">
@@ -28006,7 +28021,7 @@
       </c>
       <c r="W114" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X114" t="inlineStr">
@@ -28136,6 +28151,11 @@
           <t>2022</t>
         </is>
       </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="AQ115" t="inlineStr">
         <is>
           <t>2025</t>
@@ -28285,7 +28305,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X116" t="inlineStr">
@@ -28539,7 +28559,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
@@ -28802,7 +28822,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X118" t="inlineStr">
@@ -29079,7 +29099,7 @@
       </c>
       <c r="W119" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X119" t="inlineStr">
@@ -29366,7 +29386,7 @@
       </c>
       <c r="W120" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X120" t="inlineStr">
@@ -29660,7 +29680,7 @@
       </c>
       <c r="W121" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X121" t="inlineStr">
@@ -29877,7 +29897,7 @@
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="Z122" t="inlineStr">
@@ -30069,7 +30089,7 @@
       </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="Y123" t="inlineStr">
@@ -30308,7 +30328,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -30526,7 +30546,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -30769,7 +30789,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X126" t="inlineStr">
@@ -31056,7 +31076,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
@@ -31343,7 +31363,7 @@
       </c>
       <c r="W128" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X128" t="inlineStr">
@@ -31640,7 +31660,7 @@
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X129" t="inlineStr">
@@ -31864,7 +31884,7 @@
       </c>
       <c r="W130" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X130" t="inlineStr">
@@ -32087,7 +32107,7 @@
       </c>
       <c r="W131" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X131" t="inlineStr">
@@ -32340,7 +32360,7 @@
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X132" t="inlineStr">
@@ -32542,7 +32562,7 @@
       </c>
       <c r="W133" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="AC133" t="inlineStr">
@@ -32687,7 +32707,7 @@
       </c>
       <c r="W134" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X134" t="inlineStr">
@@ -32925,7 +32945,7 @@
       </c>
       <c r="W135" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X135" t="inlineStr">
@@ -33200,7 +33220,7 @@
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X136" t="inlineStr">
@@ -33489,7 +33509,7 @@
       </c>
       <c r="W137" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X137" t="inlineStr">
@@ -33793,7 +33813,7 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X138" t="inlineStr">
@@ -34037,7 +34057,7 @@
       </c>
       <c r="W139" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X139" t="inlineStr">
@@ -34275,7 +34295,7 @@
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X140" t="inlineStr">
@@ -34498,7 +34518,7 @@
       </c>
       <c r="W141" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X141" t="inlineStr">
@@ -34718,7 +34738,7 @@
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X142" t="inlineStr">
@@ -34986,7 +35006,7 @@
       </c>
       <c r="W143" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X143" t="inlineStr">
@@ -35225,7 +35245,7 @@
       </c>
       <c r="W144" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X144" t="inlineStr">
@@ -35498,7 +35518,7 @@
       </c>
       <c r="W145" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X145" t="inlineStr">
@@ -35752,7 +35772,7 @@
       </c>
       <c r="W146" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X146" t="inlineStr">
@@ -35968,7 +35988,7 @@
       </c>
       <c r="W147" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X147" t="inlineStr">
@@ -36131,7 +36151,7 @@
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X148" t="inlineStr">
@@ -36309,7 +36329,7 @@
       </c>
       <c r="W149" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X149" t="inlineStr">
@@ -36492,7 +36512,7 @@
       </c>
       <c r="W150" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X150" t="inlineStr">
@@ -36638,6 +36658,11 @@
           <t>2022</t>
         </is>
       </c>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="AC151" t="inlineStr">
         <is>
           <t>2022</t>
@@ -36780,7 +36805,7 @@
       </c>
       <c r="W152" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X152" t="inlineStr">
@@ -36998,7 +37023,7 @@
       </c>
       <c r="W153" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X153" t="inlineStr">
@@ -37261,7 +37286,7 @@
       </c>
       <c r="W154" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X154" t="inlineStr">
@@ -37558,7 +37583,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X155" t="inlineStr">
@@ -37802,7 +37827,7 @@
       </c>
       <c r="W156" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X156" t="inlineStr">
@@ -38045,7 +38070,7 @@
       </c>
       <c r="W157" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X157" t="inlineStr">
@@ -38267,7 +38292,7 @@
       </c>
       <c r="W158" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X158" t="inlineStr">
@@ -38442,7 +38467,7 @@
       </c>
       <c r="W159" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X159" t="inlineStr">
@@ -38670,7 +38695,7 @@
       </c>
       <c r="W160" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X160" t="inlineStr">
@@ -38883,7 +38908,7 @@
       </c>
       <c r="W161" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X161" t="inlineStr">
@@ -39121,7 +39146,7 @@
       </c>
       <c r="W162" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X162" t="inlineStr">
@@ -39383,7 +39408,7 @@
       </c>
       <c r="W163" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X163" t="inlineStr">
@@ -39620,11 +39645,6 @@
           <t>2022</t>
         </is>
       </c>
-      <c r="W164" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
       <c r="X164" t="inlineStr">
         <is>
           <t>2023</t>
@@ -39830,7 +39850,7 @@
       </c>
       <c r="W165" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X165" t="inlineStr">
@@ -40103,7 +40123,7 @@
       </c>
       <c r="W166" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X166" t="inlineStr">
@@ -40353,11 +40373,6 @@
           <t>2022</t>
         </is>
       </c>
-      <c r="W167" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
       <c r="X167" t="inlineStr">
         <is>
           <t>2023</t>
@@ -40608,7 +40623,7 @@
       </c>
       <c r="W168" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X168" t="inlineStr">
@@ -40821,7 +40836,7 @@
       </c>
       <c r="W169" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X169" t="inlineStr">
@@ -41079,7 +41094,7 @@
       </c>
       <c r="W170" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X170" t="inlineStr">
@@ -41303,7 +41318,7 @@
       </c>
       <c r="W171" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X171" t="inlineStr">
@@ -41559,7 +41574,7 @@
       </c>
       <c r="W172" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X172" t="inlineStr">
@@ -41828,7 +41843,7 @@
       </c>
       <c r="W173" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X173" t="inlineStr">
@@ -42067,7 +42082,7 @@
       </c>
       <c r="W174" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X174" t="inlineStr">
@@ -42335,7 +42350,7 @@
       </c>
       <c r="W175" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X175" t="inlineStr">
@@ -42572,7 +42587,7 @@
       </c>
       <c r="W176" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X176" t="inlineStr">
@@ -42767,7 +42782,7 @@
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X177" t="inlineStr">
@@ -43020,7 +43035,7 @@
       </c>
       <c r="W178" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X178" t="inlineStr">
@@ -43297,7 +43312,7 @@
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X179" t="inlineStr">
@@ -43546,7 +43561,7 @@
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X180" t="inlineStr">
@@ -43711,7 +43726,7 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="Z181" t="inlineStr">
@@ -43913,7 +43928,7 @@
       </c>
       <c r="W182" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X182" t="inlineStr">
@@ -44195,7 +44210,7 @@
       </c>
       <c r="W183" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X183" t="inlineStr">
@@ -44442,7 +44457,7 @@
       </c>
       <c r="W184" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X184" t="inlineStr">
@@ -44635,7 +44650,7 @@
       </c>
       <c r="W185" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X185" t="inlineStr">
@@ -44913,7 +44928,7 @@
       </c>
       <c r="W186" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X186" t="inlineStr">
@@ -45205,7 +45220,7 @@
       </c>
       <c r="W187" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X187" t="inlineStr">
@@ -45454,7 +45469,7 @@
       </c>
       <c r="W188" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X188" t="inlineStr">
@@ -45732,7 +45747,7 @@
       </c>
       <c r="W189" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X189" t="inlineStr">
@@ -45949,7 +45964,7 @@
       </c>
       <c r="W190" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X190" t="inlineStr">
@@ -46177,7 +46192,7 @@
       </c>
       <c r="W191" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X191" t="inlineStr">
@@ -46436,7 +46451,7 @@
       </c>
       <c r="W192" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X192" t="inlineStr">
@@ -46710,7 +46725,7 @@
       </c>
       <c r="W193" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X193" t="inlineStr">
@@ -46997,7 +47012,7 @@
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X194" t="inlineStr">
@@ -47289,7 +47304,7 @@
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="X195" t="inlineStr">

</xml_diff>